<commit_message>
Extend Q2 time frontier to verified 23-25 sorties
</commit_message>
<xml_diff>
--- a/results_q2_time/selection/q2_time_result_template.xlsx
+++ b/results_q2_time/selection/q2_time_result_template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1_单点组批" sheetId="1" r:id="R4efc907c42064ece"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2_运输架次" sheetId="2" r:id="Rf5fedb3d878a4b62"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2_逐箱交付" sheetId="3" r:id="R43d9c74c5737480a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_中继架次" sheetId="4" r:id="R99c6e07d1a654e4a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_通信保障" sheetId="5" r:id="R005027f50c3246b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_分区配置" sheetId="6" r:id="Rdecd8f16bf1b499f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q1_单点组批" sheetId="1" r:id="R276908387be14b7c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2_运输架次" sheetId="2" r:id="R4d9c789ed89d456f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q2_逐箱交付" sheetId="3" r:id="R7bc82ef2c3084583"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_中继架次" sheetId="4" r:id="R2ac84e8291e24643"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q3_通信保障" sheetId="5" r:id="R3873bb71919940ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Q4_分区配置" sheetId="6" r:id="R138de9e60c954c50"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1536,13 +1536,13 @@
         <x:v>T001</x:v>
       </x:c>
       <x:c r="B2" s="4" t="str">
-        <x:v>U08</x:v>
+        <x:v>U07</x:v>
       </x:c>
       <x:c r="C2" s="4" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="D2" s="4" t="str">
-        <x:v>C03</x:v>
+        <x:v>C04</x:v>
       </x:c>
       <x:c r="E2" s="4" t="n">
         <x:v>0</x:v>
@@ -1559,189 +1559,189 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="4" t="str">
-        <x:v>T003</x:v>
+        <x:v>T002</x:v>
       </x:c>
       <x:c r="B3" s="4" t="str">
-        <x:v>U03</x:v>
+        <x:v>U06</x:v>
       </x:c>
       <x:c r="C3" s="4" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D3" s="4" t="str">
-        <x:v>A01</x:v>
+        <x:v>B01</x:v>
       </x:c>
       <x:c r="E3" s="4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F3" s="4" t="str">
-        <x:v>S013</x:v>
+        <x:v>S006</x:v>
       </x:c>
       <x:c r="G3" s="4" t="n">
-        <x:v>1602.592736</x:v>
+        <x:v>1269.979917</x:v>
       </x:c>
       <x:c r="H3" s="4" t="n">
-        <x:v>1.953925</x:v>
+        <x:v>1.223874</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>T004</x:v>
+        <x:v>T003</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>U07</x:v>
+        <x:v>U04</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>C</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>C02</x:v>
+        <x:v>A06</x:v>
       </x:c>
       <x:c r="E4" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>S001</x:v>
+        <x:v>S013</x:v>
       </x:c>
       <x:c r="G4" t="n">
-        <x:v>1495.426178</x:v>
+        <x:v>1602.592736</x:v>
       </x:c>
       <x:c r="H4" t="n">
-        <x:v>2.672703</x:v>
+        <x:v>1.953925</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>T005</x:v>
+        <x:v>T004</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>U04</x:v>
+        <x:v>U08</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>A</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>A06</x:v>
+        <x:v>C03</x:v>
       </x:c>
       <x:c r="E5" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>S009→S002</x:v>
+        <x:v>S001</x:v>
       </x:c>
       <x:c r="G5" t="n">
-        <x:v>2281.459959</x:v>
+        <x:v>1429.426178</x:v>
       </x:c>
       <x:c r="H5" t="n">
-        <x:v>3.00442</x:v>
+        <x:v>2.528666</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>T007</x:v>
+        <x:v>T005</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>U02</x:v>
+        <x:v>U03</x:v>
       </x:c>
       <x:c r="C6" t="str">
         <x:v>A</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>A04</x:v>
+        <x:v>A05</x:v>
       </x:c>
       <x:c r="E6" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>S001</x:v>
+        <x:v>S012</x:v>
       </x:c>
       <x:c r="G6" t="n">
-        <x:v>1312.470877</x:v>
+        <x:v>2130.639089</x:v>
       </x:c>
       <x:c r="H6" t="n">
-        <x:v>1.268023</x:v>
+        <x:v>2.969256</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>T008</x:v>
+        <x:v>T006</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>U06</x:v>
+        <x:v>U02</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>B04</x:v>
+        <x:v>A04</x:v>
       </x:c>
       <x:c r="E7" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>S011</x:v>
+        <x:v>S001</x:v>
       </x:c>
       <x:c r="G7" t="n">
-        <x:v>1189.630286</x:v>
+        <x:v>1312.470877</x:v>
       </x:c>
       <x:c r="H7" t="n">
-        <x:v>1.077171</x:v>
+        <x:v>1.268023</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
-        <x:v>T010</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>U01</x:v>
+        <x:v>U05</x:v>
       </x:c>
       <x:c r="C8" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>A02</x:v>
+        <x:v>B04</x:v>
       </x:c>
       <x:c r="E8" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F8" t="str">
-        <x:v>S003→S015</x:v>
+        <x:v>S010</x:v>
       </x:c>
       <x:c r="G8" t="n">
-        <x:v>2608.040897</x:v>
+        <x:v>1554.571359</x:v>
       </x:c>
       <x:c r="H8" t="n">
-        <x:v>3.299758</x:v>
+        <x:v>1.821045</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" t="str">
-        <x:v>T012</x:v>
+        <x:v>T014</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>U05</x:v>
+        <x:v>U01</x:v>
       </x:c>
       <x:c r="C9" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>B02</x:v>
+        <x:v>A02</x:v>
       </x:c>
       <x:c r="E9" t="n">
         <x:v>0</x:v>
       </x:c>
       <x:c r="F9" t="str">
-        <x:v>S014→S010</x:v>
+        <x:v>S009→S002</x:v>
       </x:c>
       <x:c r="G9" t="n">
-        <x:v>2107.280973</x:v>
+        <x:v>2281.459959</x:v>
       </x:c>
       <x:c r="H9" t="n">
-        <x:v>2.322729</x:v>
+        <x:v>3.00442</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
       <x:c r="A10" t="str">
-        <x:v>T002</x:v>
+        <x:v>T009</x:v>
       </x:c>
       <x:c r="B10" t="str">
         <x:v>U06</x:v>
@@ -1750,24 +1750,24 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>B01</x:v>
+        <x:v>B02</x:v>
       </x:c>
       <x:c r="E10" t="n">
-        <x:v>1189.630286</x:v>
+        <x:v>1269.979917</x:v>
       </x:c>
       <x:c r="F10" t="str">
-        <x:v>S006</x:v>
+        <x:v>S011</x:v>
       </x:c>
       <x:c r="G10" t="n">
         <x:v>2459.610203</x:v>
       </x:c>
       <x:c r="H10" t="n">
-        <x:v>1.223874</x:v>
+        <x:v>1.077171</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" t="str">
-        <x:v>T011</x:v>
+        <x:v>T015</x:v>
       </x:c>
       <x:c r="B11" t="str">
         <x:v>U02</x:v>
@@ -1776,7 +1776,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>A03</x:v>
+        <x:v>A01</x:v>
       </x:c>
       <x:c r="E11" t="n">
         <x:v>1312.470877</x:v>
@@ -1793,25 +1793,25 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>U07</x:v>
+        <x:v>U08</x:v>
       </x:c>
       <x:c r="C12" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>C01</x:v>
+        <x:v>C02</x:v>
       </x:c>
       <x:c r="E12" t="n">
-        <x:v>1495.426178</x:v>
+        <x:v>1429.426178</x:v>
       </x:c>
       <x:c r="F12" t="str">
         <x:v>S006→S007</x:v>
       </x:c>
       <x:c r="G12" t="n">
-        <x:v>3834.02406</x:v>
+        <x:v>3768.02406</x:v>
       </x:c>
       <x:c r="H12" t="n">
         <x:v>4.075608</x:v>
@@ -1819,16 +1819,16 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>U08</x:v>
+        <x:v>U07</x:v>
       </x:c>
       <x:c r="C13" t="str">
         <x:v>C</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>C04</x:v>
+        <x:v>C01</x:v>
       </x:c>
       <x:c r="E13" t="n">
         <x:v>1495.426178</x:v>
@@ -1845,62 +1845,62 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" t="str">
-        <x:v>T006</x:v>
+        <x:v>T013</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>U03</x:v>
+        <x:v>U05</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>A</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>A05</x:v>
+        <x:v>B03</x:v>
       </x:c>
       <x:c r="E14" t="n">
-        <x:v>1602.592736</x:v>
+        <x:v>1554.571359</x:v>
       </x:c>
       <x:c r="F14" t="str">
-        <x:v>S012</x:v>
+        <x:v>S014</x:v>
       </x:c>
       <x:c r="G14" t="n">
-        <x:v>3733.231825</x:v>
+        <x:v>3399.110249</x:v>
       </x:c>
       <x:c r="H14" t="n">
-        <x:v>2.969256</x:v>
+        <x:v>2.127681</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" t="str">
-        <x:v>T016</x:v>
+        <x:v>T022</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>U05</x:v>
+        <x:v>U04</x:v>
       </x:c>
       <x:c r="C15" t="str">
-        <x:v>B</x:v>
+        <x:v>A</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>B03</x:v>
+        <x:v>A03</x:v>
       </x:c>
       <x:c r="E15" t="n">
-        <x:v>2107.280973</x:v>
+        <x:v>1602.592736</x:v>
       </x:c>
       <x:c r="F15" t="str">
-        <x:v>S008</x:v>
+        <x:v>S015</x:v>
       </x:c>
       <x:c r="G15" t="n">
-        <x:v>4065.322245</x:v>
+        <x:v>3572.802583</x:v>
       </x:c>
       <x:c r="H15" t="n">
-        <x:v>2.982875</x:v>
+        <x:v>2.561541</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
       <x:c r="A16" t="str">
-        <x:v>T015</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>U04</x:v>
+        <x:v>U03</x:v>
       </x:c>
       <x:c r="C16" t="str">
         <x:v>A</x:v>
@@ -1909,21 +1909,21 @@
         <x:v>A04</x:v>
       </x:c>
       <x:c r="E16" t="n">
-        <x:v>2281.459959</x:v>
+        <x:v>2178.788712</x:v>
       </x:c>
       <x:c r="F16" t="str">
-        <x:v>S005→S004</x:v>
+        <x:v>S003→S015</x:v>
       </x:c>
       <x:c r="G16" t="n">
-        <x:v>4762.409374</x:v>
+        <x:v>4786.829609</x:v>
       </x:c>
       <x:c r="H16" t="n">
-        <x:v>3.142786</x:v>
+        <x:v>3.299758</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
       <x:c r="A17" t="str">
-        <x:v>T009</x:v>
+        <x:v>T018</x:v>
       </x:c>
       <x:c r="B17" t="str">
         <x:v>U06</x:v>
@@ -1932,24 +1932,24 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>B04</x:v>
+        <x:v>B01</x:v>
       </x:c>
       <x:c r="E17" t="n">
-        <x:v>2459.610203</x:v>
+        <x:v>2466.992001</x:v>
       </x:c>
       <x:c r="F17" t="str">
-        <x:v>S010→S014</x:v>
+        <x:v>S008</x:v>
       </x:c>
       <x:c r="G17" t="n">
-        <x:v>4566.891176</x:v>
+        <x:v>4425.033273</x:v>
       </x:c>
       <x:c r="H17" t="n">
-        <x:v>2.265766</x:v>
+        <x:v>2.982875</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
       <x:c r="A18" t="str">
-        <x:v>T024</x:v>
+        <x:v>T023</x:v>
       </x:c>
       <x:c r="B18" t="str">
         <x:v>U01</x:v>
@@ -1958,7 +1958,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>A01</x:v>
+        <x:v>A06</x:v>
       </x:c>
       <x:c r="E18" t="n">
         <x:v>2667.059898</x:v>
@@ -1975,33 +1975,33 @@
     </x:row>
     <x:row r="19">
       <x:c r="A19" t="str">
-        <x:v>T019</x:v>
+        <x:v>T016</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>U08</x:v>
+        <x:v>U05</x:v>
       </x:c>
       <x:c r="C19" t="str">
-        <x:v>C</x:v>
+        <x:v>B</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>C02</x:v>
+        <x:v>B04</x:v>
       </x:c>
       <x:c r="E19" t="n">
-        <x:v>3610.507819</x:v>
+        <x:v>3399.110249</x:v>
       </x:c>
       <x:c r="F19" t="str">
-        <x:v>S003</x:v>
+        <x:v>S008</x:v>
       </x:c>
       <x:c r="G19" t="n">
-        <x:v>6046.31734</x:v>
+        <x:v>5297.151521</x:v>
       </x:c>
       <x:c r="H19" t="n">
-        <x:v>6.14777</x:v>
+        <x:v>2.77042</x:v>
       </x:c>
     </x:row>
     <x:row r="20">
       <x:c r="A20" t="str">
-        <x:v>T017</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="B20" t="str">
         <x:v>U02</x:v>
@@ -2010,24 +2010,24 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>A06</x:v>
+        <x:v>A05</x:v>
       </x:c>
       <x:c r="E20" t="n">
-        <x:v>3649.403581</x:v>
+        <x:v>3488.424084</x:v>
       </x:c>
       <x:c r="F20" t="str">
-        <x:v>S013→S012</x:v>
+        <x:v>S005→S004</x:v>
       </x:c>
       <x:c r="G20" t="n">
-        <x:v>5993.250655</x:v>
+        <x:v>5969.373499</x:v>
       </x:c>
       <x:c r="H20" t="n">
-        <x:v>2.98926</x:v>
+        <x:v>3.142786</x:v>
       </x:c>
     </x:row>
     <x:row r="21">
       <x:c r="A21" t="str">
-        <x:v>T025</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="B21" t="str">
         <x:v>U07</x:v>
@@ -2036,27 +2036,27 @@
         <x:v>C</x:v>
       </x:c>
       <x:c r="D21" t="str">
-        <x:v>C03</x:v>
+        <x:v>C04</x:v>
       </x:c>
       <x:c r="E21" t="n">
-        <x:v>3834.02406</x:v>
+        <x:v>3610.507819</x:v>
       </x:c>
       <x:c r="F21" t="str">
-        <x:v>S004</x:v>
+        <x:v>S003</x:v>
       </x:c>
       <x:c r="G21" t="n">
-        <x:v>6073.208125</x:v>
+        <x:v>6046.31734</x:v>
       </x:c>
       <x:c r="H21" t="n">
-        <x:v>6.038195</x:v>
+        <x:v>6.14777</x:v>
       </x:c>
     </x:row>
     <x:row r="22">
       <x:c r="A22" t="str">
-        <x:v>T021</x:v>
+        <x:v>T019</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>U03</x:v>
+        <x:v>U04</x:v>
       </x:c>
       <x:c r="C22" t="str">
         <x:v>A</x:v>
@@ -2065,47 +2065,47 @@
         <x:v>A02</x:v>
       </x:c>
       <x:c r="E22" t="n">
-        <x:v>4061.30436</x:v>
+        <x:v>3649.403581</x:v>
       </x:c>
       <x:c r="F22" t="str">
-        <x:v>S015</x:v>
+        <x:v>S013→S012</x:v>
       </x:c>
       <x:c r="G22" t="n">
-        <x:v>6031.514207</x:v>
+        <x:v>5993.250655</x:v>
       </x:c>
       <x:c r="H22" t="n">
-        <x:v>2.561541</x:v>
+        <x:v>2.98926</x:v>
       </x:c>
     </x:row>
     <x:row r="23">
       <x:c r="A23" t="str">
-        <x:v>T022</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>U05</x:v>
+        <x:v>U08</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>B</x:v>
+        <x:v>C</x:v>
       </x:c>
       <x:c r="D23" t="str">
-        <x:v>B02</x:v>
+        <x:v>C03</x:v>
       </x:c>
       <x:c r="E23" t="n">
-        <x:v>4065.322245</x:v>
+        <x:v>3768.02406</x:v>
       </x:c>
       <x:c r="F23" t="str">
-        <x:v>S008</x:v>
+        <x:v>S004</x:v>
       </x:c>
       <x:c r="G23" t="n">
-        <x:v>5963.363516</x:v>
+        <x:v>6007.208125</x:v>
       </x:c>
       <x:c r="H23" t="n">
-        <x:v>2.77042</x:v>
+        <x:v>6.038195</x:v>
       </x:c>
     </x:row>
     <x:row r="24">
       <x:c r="A24" t="str">
-        <x:v>T020</x:v>
+        <x:v>T010</x:v>
       </x:c>
       <x:c r="B24" t="str">
         <x:v>U01</x:v>
@@ -2114,7 +2114,7 @@
         <x:v>A</x:v>
       </x:c>
       <x:c r="D24" t="str">
-        <x:v>A03</x:v>
+        <x:v>A01</x:v>
       </x:c>
       <x:c r="E24" t="n">
         <x:v>4358.594384</x:v>
@@ -2131,7 +2131,7 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
-        <x:v>T018</x:v>
+        <x:v>T024</x:v>
       </x:c>
       <x:c r="B25" t="str">
         <x:v>U06</x:v>
@@ -2140,19 +2140,45 @@
         <x:v>B</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>B01</x:v>
+        <x:v>B02</x:v>
       </x:c>
       <x:c r="E25" t="n">
-        <x:v>4566.891176</x:v>
+        <x:v>4425.033273</x:v>
       </x:c>
       <x:c r="F25" t="str">
         <x:v>S005</x:v>
       </x:c>
       <x:c r="G25" t="n">
-        <x:v>6085.91552</x:v>
+        <x:v>5944.057617</x:v>
       </x:c>
       <x:c r="H25" t="n">
         <x:v>1.841574</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
+        <x:v>T025</x:v>
+      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>U03</x:v>
+      </x:c>
+      <x:c r="C26" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D26" t="str">
+        <x:v>A03</x:v>
+      </x:c>
+      <x:c r="E26" t="n">
+        <x:v>4812.803234</x:v>
+      </x:c>
+      <x:c r="F26" t="str">
+        <x:v>S001</x:v>
+      </x:c>
+      <x:c r="G26" t="n">
+        <x:v>6005.274111</x:v>
+      </x:c>
+      <x:c r="H26" t="n">
+        <x:v>1.181509</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2231,13 +2257,13 @@
         <x:v>S001-HYG-01</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>T004</x:v>
+        <x:v>T025</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>5662.162006</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -2251,7 +2277,7 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>1116.898089</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -2259,7 +2285,7 @@
         <x:v>S001-MED-01</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>T007</x:v>
+        <x:v>T006</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>S001</x:v>
@@ -2273,7 +2299,7 @@
         <x:v>S001-MED-02</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>T007</x:v>
+        <x:v>T006</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>S001</x:v>
@@ -2287,7 +2313,7 @@
         <x:v>S001-WAT-01</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>T007</x:v>
+        <x:v>T006</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>S001</x:v>
@@ -2307,7 +2333,7 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D10" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>1116.898089</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2321,7 +2347,7 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D11" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>1116.898089</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2335,7 +2361,7 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D12" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>1116.898089</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2349,7 +2375,7 @@
         <x:v>S001</x:v>
       </x:c>
       <x:c r="D13" t="n">
-        <x:v>1182.898089</x:v>
+        <x:v>1116.898089</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2399,7 +2425,7 @@
         <x:v>S002-FOD-01</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C17" t="str">
         <x:v>S002</x:v>
@@ -2413,7 +2439,7 @@
         <x:v>S002-FOD-02</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>S002</x:v>
@@ -2427,7 +2453,7 @@
         <x:v>S002-HYG-01</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>S002</x:v>
@@ -2441,7 +2467,7 @@
         <x:v>S002-MED-01</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>T005</x:v>
+        <x:v>T014</x:v>
       </x:c>
       <x:c r="C20" t="str">
         <x:v>S002</x:v>
@@ -2455,7 +2481,7 @@
         <x:v>S002-WAT-01</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>T005</x:v>
+        <x:v>T014</x:v>
       </x:c>
       <x:c r="C21" t="str">
         <x:v>S002</x:v>
@@ -2469,7 +2495,7 @@
         <x:v>S002-WAT-02</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C22" t="str">
         <x:v>S002</x:v>
@@ -2483,7 +2509,7 @@
         <x:v>S002-WAT-03</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C23" t="str">
         <x:v>S002</x:v>
@@ -2497,7 +2523,7 @@
         <x:v>S002-WAT-04</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>T014</x:v>
+        <x:v>T012</x:v>
       </x:c>
       <x:c r="C24" t="str">
         <x:v>S002</x:v>
@@ -2511,7 +2537,7 @@
         <x:v>S003-FOD-01</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C25" t="str">
         <x:v>S003</x:v>
@@ -2525,7 +2551,7 @@
         <x:v>S003-FOD-02</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C26" t="str">
         <x:v>S003</x:v>
@@ -2539,7 +2565,7 @@
         <x:v>S003-HYG-01</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C27" t="str">
         <x:v>S003</x:v>
@@ -2553,13 +2579,13 @@
         <x:v>S003-MED-01</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>T010</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="C28" t="str">
         <x:v>S003</x:v>
       </x:c>
       <x:c r="D28" t="n">
-        <x:v>1439.11183</x:v>
+        <x:v>3617.900542</x:v>
       </x:c>
     </x:row>
     <x:row r="29">
@@ -2567,13 +2593,13 @@
         <x:v>S003-WAT-01</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>T010</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="C29" t="str">
         <x:v>S003</x:v>
       </x:c>
       <x:c r="D29" t="n">
-        <x:v>1439.11183</x:v>
+        <x:v>3617.900542</x:v>
       </x:c>
     </x:row>
     <x:row r="30">
@@ -2581,7 +2607,7 @@
         <x:v>S003-WAT-02</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C30" t="str">
         <x:v>S003</x:v>
@@ -2595,7 +2621,7 @@
         <x:v>S003-WAT-03</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C31" t="str">
         <x:v>S003</x:v>
@@ -2609,7 +2635,7 @@
         <x:v>S003-WAT-04</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>T019</x:v>
+        <x:v>T020</x:v>
       </x:c>
       <x:c r="C32" t="str">
         <x:v>S003</x:v>
@@ -2623,13 +2649,13 @@
         <x:v>S004-FOD-01</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>T025</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="C33" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D33" t="n">
-        <x:v>5353.586093</x:v>
+        <x:v>5287.586093</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -2637,13 +2663,13 @@
         <x:v>S004-HYG-01</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>T025</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="C34" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D34" t="n">
-        <x:v>5353.586093</x:v>
+        <x:v>5287.586093</x:v>
       </x:c>
     </x:row>
     <x:row r="35">
@@ -2651,13 +2677,13 @@
         <x:v>S004-MED-01</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>T015</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="C35" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D35" t="n">
-        <x:v>3952.07634</x:v>
+        <x:v>5159.040465</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -2665,13 +2691,13 @@
         <x:v>S004-WAT-01</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>T025</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="C36" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D36" t="n">
-        <x:v>5353.586093</x:v>
+        <x:v>5287.586093</x:v>
       </x:c>
     </x:row>
     <x:row r="37">
@@ -2679,13 +2705,13 @@
         <x:v>S004-WAT-02</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>T025</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="C37" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D37" t="n">
-        <x:v>5353.586093</x:v>
+        <x:v>5287.586093</x:v>
       </x:c>
     </x:row>
     <x:row r="38">
@@ -2693,13 +2719,13 @@
         <x:v>S004-WAT-03</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>T025</x:v>
+        <x:v>T021</x:v>
       </x:c>
       <x:c r="C38" t="str">
         <x:v>S004</x:v>
       </x:c>
       <x:c r="D38" t="n">
-        <x:v>5353.586093</x:v>
+        <x:v>5287.586093</x:v>
       </x:c>
     </x:row>
     <x:row r="39">
@@ -2707,7 +2733,7 @@
         <x:v>S005-FOD-01</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>T020</x:v>
+        <x:v>T010</x:v>
       </x:c>
       <x:c r="C39" t="str">
         <x:v>S005</x:v>
@@ -2721,13 +2747,13 @@
         <x:v>S005-HYG-01</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>T018</x:v>
+        <x:v>T024</x:v>
       </x:c>
       <x:c r="C40" t="str">
         <x:v>S005</x:v>
       </x:c>
       <x:c r="D40" t="n">
-        <x:v>5609.160015</x:v>
+        <x:v>5467.302112</x:v>
       </x:c>
     </x:row>
     <x:row r="41">
@@ -2735,13 +2761,13 @@
         <x:v>S005-MED-01</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>T015</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="C41" t="str">
         <x:v>S005</x:v>
       </x:c>
       <x:c r="D41" t="n">
-        <x:v>3442.095678</x:v>
+        <x:v>4649.059803</x:v>
       </x:c>
     </x:row>
     <x:row r="42">
@@ -2749,13 +2775,13 @@
         <x:v>S005-WAT-01</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>T015</x:v>
+        <x:v>T008</x:v>
       </x:c>
       <x:c r="C42" t="str">
         <x:v>S005</x:v>
       </x:c>
       <x:c r="D42" t="n">
-        <x:v>3442.095678</x:v>
+        <x:v>4649.059803</x:v>
       </x:c>
     </x:row>
     <x:row r="43">
@@ -2763,7 +2789,7 @@
         <x:v>S005-WAT-02</x:v>
       </x:c>
       <x:c r="B43" t="str">
-        <x:v>T020</x:v>
+        <x:v>T010</x:v>
       </x:c>
       <x:c r="C43" t="str">
         <x:v>S005</x:v>
@@ -2777,13 +2803,13 @@
         <x:v>S005-WAT-03</x:v>
       </x:c>
       <x:c r="B44" t="str">
-        <x:v>T018</x:v>
+        <x:v>T024</x:v>
       </x:c>
       <x:c r="C44" t="str">
         <x:v>S005</x:v>
       </x:c>
       <x:c r="D44" t="n">
-        <x:v>5609.160015</x:v>
+        <x:v>5467.302112</x:v>
       </x:c>
     </x:row>
     <x:row r="45">
@@ -2797,7 +2823,7 @@
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D45" t="n">
-        <x:v>2133.383578</x:v>
+        <x:v>943.753292</x:v>
       </x:c>
     </x:row>
     <x:row r="46">
@@ -2805,13 +2831,13 @@
         <x:v>S006-HYG-01</x:v>
       </x:c>
       <x:c r="B46" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C46" t="str">
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D46" t="n">
-        <x:v>2598.588719</x:v>
+        <x:v>2532.588719</x:v>
       </x:c>
     </x:row>
     <x:row r="47">
@@ -2825,7 +2851,7 @@
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D47" t="n">
-        <x:v>2133.383578</x:v>
+        <x:v>943.753292</x:v>
       </x:c>
     </x:row>
     <x:row r="48">
@@ -2839,7 +2865,7 @@
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D48" t="n">
-        <x:v>2133.383578</x:v>
+        <x:v>943.753292</x:v>
       </x:c>
     </x:row>
     <x:row r="49">
@@ -2847,13 +2873,13 @@
         <x:v>S006-WAT-02</x:v>
       </x:c>
       <x:c r="B49" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C49" t="str">
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D49" t="n">
-        <x:v>2598.588719</x:v>
+        <x:v>2532.588719</x:v>
       </x:c>
     </x:row>
     <x:row r="50">
@@ -2861,13 +2887,13 @@
         <x:v>S006-WAT-03</x:v>
       </x:c>
       <x:c r="B50" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C50" t="str">
         <x:v>S006</x:v>
       </x:c>
       <x:c r="D50" t="n">
-        <x:v>2598.588719</x:v>
+        <x:v>2532.588719</x:v>
       </x:c>
     </x:row>
     <x:row r="51">
@@ -2875,13 +2901,13 @@
         <x:v>S007-FOD-01</x:v>
       </x:c>
       <x:c r="B51" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C51" t="str">
         <x:v>S007</x:v>
       </x:c>
       <x:c r="D51" t="n">
-        <x:v>3283.371857</x:v>
+        <x:v>3217.371857</x:v>
       </x:c>
     </x:row>
     <x:row r="52">
@@ -2889,13 +2915,13 @@
         <x:v>S007-HYG-01</x:v>
       </x:c>
       <x:c r="B52" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C52" t="str">
         <x:v>S007</x:v>
       </x:c>
       <x:c r="D52" t="n">
-        <x:v>3283.371857</x:v>
+        <x:v>3217.371857</x:v>
       </x:c>
     </x:row>
     <x:row r="53">
@@ -2903,7 +2929,7 @@
         <x:v>S007-MED-01</x:v>
       </x:c>
       <x:c r="B53" t="str">
-        <x:v>T011</x:v>
+        <x:v>T015</x:v>
       </x:c>
       <x:c r="C53" t="str">
         <x:v>S007</x:v>
@@ -2917,7 +2943,7 @@
         <x:v>S007-WAT-01</x:v>
       </x:c>
       <x:c r="B54" t="str">
-        <x:v>T011</x:v>
+        <x:v>T015</x:v>
       </x:c>
       <x:c r="C54" t="str">
         <x:v>S007</x:v>
@@ -2931,13 +2957,13 @@
         <x:v>S007-WAT-02</x:v>
       </x:c>
       <x:c r="B55" t="str">
-        <x:v>T013</x:v>
+        <x:v>T011</x:v>
       </x:c>
       <x:c r="C55" t="str">
         <x:v>S007</x:v>
       </x:c>
       <x:c r="D55" t="n">
-        <x:v>3283.371857</x:v>
+        <x:v>3217.371857</x:v>
       </x:c>
     </x:row>
     <x:row r="56">
@@ -2945,13 +2971,13 @@
         <x:v>S008-FOD-01</x:v>
       </x:c>
       <x:c r="B56" t="str">
-        <x:v>T016</x:v>
+        <x:v>T018</x:v>
       </x:c>
       <x:c r="C56" t="str">
         <x:v>S008</x:v>
       </x:c>
       <x:c r="D56" t="n">
-        <x:v>3396.528275</x:v>
+        <x:v>3756.239304</x:v>
       </x:c>
     </x:row>
     <x:row r="57">
@@ -2959,13 +2985,13 @@
         <x:v>S008-HYG-01</x:v>
       </x:c>
       <x:c r="B57" t="str">
-        <x:v>T022</x:v>
+        <x:v>T016</x:v>
       </x:c>
       <x:c r="C57" t="str">
         <x:v>S008</x:v>
       </x:c>
       <x:c r="D57" t="n">
-        <x:v>5294.569547</x:v>
+        <x:v>4628.357552</x:v>
       </x:c>
     </x:row>
     <x:row r="58">
@@ -2973,13 +2999,13 @@
         <x:v>S008-MED-01</x:v>
       </x:c>
       <x:c r="B58" t="str">
-        <x:v>T016</x:v>
+        <x:v>T018</x:v>
       </x:c>
       <x:c r="C58" t="str">
         <x:v>S008</x:v>
       </x:c>
       <x:c r="D58" t="n">
-        <x:v>3396.528275</x:v>
+        <x:v>3756.239304</x:v>
       </x:c>
     </x:row>
     <x:row r="59">
@@ -2987,13 +3013,13 @@
         <x:v>S008-WAT-01</x:v>
       </x:c>
       <x:c r="B59" t="str">
-        <x:v>T016</x:v>
+        <x:v>T018</x:v>
       </x:c>
       <x:c r="C59" t="str">
         <x:v>S008</x:v>
       </x:c>
       <x:c r="D59" t="n">
-        <x:v>3396.528275</x:v>
+        <x:v>3756.239304</x:v>
       </x:c>
     </x:row>
     <x:row r="60">
@@ -3001,13 +3027,13 @@
         <x:v>S008-WAT-02</x:v>
       </x:c>
       <x:c r="B60" t="str">
-        <x:v>T022</x:v>
+        <x:v>T016</x:v>
       </x:c>
       <x:c r="C60" t="str">
         <x:v>S008</x:v>
       </x:c>
       <x:c r="D60" t="n">
-        <x:v>5294.569547</x:v>
+        <x:v>4628.357552</x:v>
       </x:c>
     </x:row>
     <x:row r="61">
@@ -3015,7 +3041,7 @@
         <x:v>S009-FOD-01</x:v>
       </x:c>
       <x:c r="B61" t="str">
-        <x:v>T024</x:v>
+        <x:v>T023</x:v>
       </x:c>
       <x:c r="C61" t="str">
         <x:v>S009</x:v>
@@ -3029,7 +3055,7 @@
         <x:v>S009-MED-01</x:v>
       </x:c>
       <x:c r="B62" t="str">
-        <x:v>T005</x:v>
+        <x:v>T014</x:v>
       </x:c>
       <x:c r="C62" t="str">
         <x:v>S009</x:v>
@@ -3043,7 +3069,7 @@
         <x:v>S009-WAT-01</x:v>
       </x:c>
       <x:c r="B63" t="str">
-        <x:v>T024</x:v>
+        <x:v>T023</x:v>
       </x:c>
       <x:c r="C63" t="str">
         <x:v>S009</x:v>
@@ -3057,13 +3083,13 @@
         <x:v>S010-FOD-01</x:v>
       </x:c>
       <x:c r="B64" t="str">
-        <x:v>T012</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="C64" t="str">
         <x:v>S010</x:v>
       </x:c>
       <x:c r="D64" t="n">
-        <x:v>1637.53196</x:v>
+        <x:v>1084.822346</x:v>
       </x:c>
     </x:row>
     <x:row r="65">
@@ -3071,13 +3097,13 @@
         <x:v>S010-MED-01</x:v>
       </x:c>
       <x:c r="B65" t="str">
-        <x:v>T009</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="C65" t="str">
         <x:v>S010</x:v>
       </x:c>
       <x:c r="D65" t="n">
-        <x:v>3514.432549</x:v>
+        <x:v>1084.822346</x:v>
       </x:c>
     </x:row>
     <x:row r="66">
@@ -3085,13 +3111,13 @@
         <x:v>S010-WAT-01</x:v>
       </x:c>
       <x:c r="B66" t="str">
-        <x:v>T009</x:v>
+        <x:v>T007</x:v>
       </x:c>
       <x:c r="C66" t="str">
         <x:v>S010</x:v>
       </x:c>
       <x:c r="D66" t="n">
-        <x:v>3514.432549</x:v>
+        <x:v>1084.822346</x:v>
       </x:c>
     </x:row>
     <x:row r="67">
@@ -3099,13 +3125,13 @@
         <x:v>S011-FOD-01</x:v>
       </x:c>
       <x:c r="B67" t="str">
-        <x:v>T008</x:v>
+        <x:v>T009</x:v>
       </x:c>
       <x:c r="C67" t="str">
         <x:v>S011</x:v>
       </x:c>
       <x:c r="D67" t="n">
-        <x:v>907.00181</x:v>
+        <x:v>2176.981727</x:v>
       </x:c>
     </x:row>
     <x:row r="68">
@@ -3113,13 +3139,13 @@
         <x:v>S011-MED-01</x:v>
       </x:c>
       <x:c r="B68" t="str">
-        <x:v>T008</x:v>
+        <x:v>T009</x:v>
       </x:c>
       <x:c r="C68" t="str">
         <x:v>S011</x:v>
       </x:c>
       <x:c r="D68" t="n">
-        <x:v>907.00181</x:v>
+        <x:v>2176.981727</x:v>
       </x:c>
     </x:row>
     <x:row r="69">
@@ -3127,13 +3153,13 @@
         <x:v>S011-WAT-01</x:v>
       </x:c>
       <x:c r="B69" t="str">
-        <x:v>T008</x:v>
+        <x:v>T009</x:v>
       </x:c>
       <x:c r="C69" t="str">
         <x:v>S011</x:v>
       </x:c>
       <x:c r="D69" t="n">
-        <x:v>907.00181</x:v>
+        <x:v>2176.981727</x:v>
       </x:c>
     </x:row>
     <x:row r="70">
@@ -3141,7 +3167,7 @@
         <x:v>S012-FOD-01</x:v>
       </x:c>
       <x:c r="B70" t="str">
-        <x:v>T017</x:v>
+        <x:v>T019</x:v>
       </x:c>
       <x:c r="C70" t="str">
         <x:v>S012</x:v>
@@ -3155,13 +3181,13 @@
         <x:v>S012-MED-01</x:v>
       </x:c>
       <x:c r="B71" t="str">
-        <x:v>T006</x:v>
+        <x:v>T005</x:v>
       </x:c>
       <x:c r="C71" t="str">
         <x:v>S012</x:v>
       </x:c>
       <x:c r="D71" t="n">
-        <x:v>2947.84228</x:v>
+        <x:v>1345.249544</x:v>
       </x:c>
     </x:row>
     <x:row r="72">
@@ -3169,13 +3195,13 @@
         <x:v>S012-WAT-01</x:v>
       </x:c>
       <x:c r="B72" t="str">
-        <x:v>T006</x:v>
+        <x:v>T005</x:v>
       </x:c>
       <x:c r="C72" t="str">
         <x:v>S012</x:v>
       </x:c>
       <x:c r="D72" t="n">
-        <x:v>2947.84228</x:v>
+        <x:v>1345.249544</x:v>
       </x:c>
     </x:row>
     <x:row r="73">
@@ -3183,7 +3209,7 @@
         <x:v>S013-FOD-01</x:v>
       </x:c>
       <x:c r="B73" t="str">
-        <x:v>T017</x:v>
+        <x:v>T019</x:v>
       </x:c>
       <x:c r="C73" t="str">
         <x:v>S013</x:v>
@@ -3225,13 +3251,13 @@
         <x:v>S014-FOD-01</x:v>
       </x:c>
       <x:c r="B76" t="str">
-        <x:v>T009</x:v>
+        <x:v>T013</x:v>
       </x:c>
       <x:c r="C76" t="str">
         <x:v>S014</x:v>
       </x:c>
       <x:c r="D76" t="n">
-        <x:v>3952.178398</x:v>
+        <x:v>2784.397471</x:v>
       </x:c>
     </x:row>
     <x:row r="77">
@@ -3239,13 +3265,13 @@
         <x:v>S014-MED-01</x:v>
       </x:c>
       <x:c r="B77" t="str">
-        <x:v>T012</x:v>
+        <x:v>T013</x:v>
       </x:c>
       <x:c r="C77" t="str">
         <x:v>S014</x:v>
       </x:c>
       <x:c r="D77" t="n">
-        <x:v>1199.826112</x:v>
+        <x:v>2784.397471</x:v>
       </x:c>
     </x:row>
     <x:row r="78">
@@ -3253,13 +3279,13 @@
         <x:v>S014-WAT-01</x:v>
       </x:c>
       <x:c r="B78" t="str">
-        <x:v>T012</x:v>
+        <x:v>T013</x:v>
       </x:c>
       <x:c r="C78" t="str">
         <x:v>S014</x:v>
       </x:c>
       <x:c r="D78" t="n">
-        <x:v>1199.826112</x:v>
+        <x:v>2784.397471</x:v>
       </x:c>
     </x:row>
     <x:row r="79">
@@ -3267,13 +3293,13 @@
         <x:v>S015-FOD-01</x:v>
       </x:c>
       <x:c r="B79" t="str">
-        <x:v>T021</x:v>
+        <x:v>T022</x:v>
       </x:c>
       <x:c r="C79" t="str">
         <x:v>S015</x:v>
       </x:c>
       <x:c r="D79" t="n">
-        <x:v>5319.849284</x:v>
+        <x:v>2861.137659</x:v>
       </x:c>
     </x:row>
     <x:row r="80">
@@ -3281,13 +3307,13 @@
         <x:v>S015-MED-01</x:v>
       </x:c>
       <x:c r="B80" t="str">
-        <x:v>T010</x:v>
+        <x:v>T017</x:v>
       </x:c>
       <x:c r="C80" t="str">
         <x:v>S015</x:v>
       </x:c>
       <x:c r="D80" t="n">
-        <x:v>1896.375974</x:v>
+        <x:v>4075.164686</x:v>
       </x:c>
     </x:row>
     <x:row r="81">
@@ -3295,13 +3321,13 @@
         <x:v>S015-WAT-01</x:v>
       </x:c>
       <x:c r="B81" t="str">
-        <x:v>T021</x:v>
+        <x:v>T022</x:v>
       </x:c>
       <x:c r="C81" t="str">
         <x:v>S015</x:v>
       </x:c>
       <x:c r="D81" t="n">
-        <x:v>5319.849284</x:v>
+        <x:v>2861.137659</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>